<commit_message>
added train results 6, 7
</commit_message>
<xml_diff>
--- a/work.xlsx
+++ b/work.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SinaOj\Documents\GitHub\Dental-XRay-YOLO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\iman_heydardoost\research_papers\dental_paper_1\Dental-XRay-YOLO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4D5E8DE-D8EB-421D-80B4-2432FABC4830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A513935-B642-478A-8CDA-3B4BD7AA3C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="15034" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="660" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dataset" sheetId="2" r:id="rId1"/>
@@ -379,10 +379,10 @@
     <t>large</t>
   </si>
   <si>
-    <t>21/2/2026</t>
-  </si>
-  <si>
     <t>xlarge</t>
+  </si>
+  <si>
+    <t>21/2/2026 rerun:28/5/2026</t>
   </si>
 </sst>
 </file>
@@ -553,7 +553,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -620,6 +620,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -912,18 +918,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA418DB5-DB83-4792-8B88-4DCE955F134C}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultColWidth="8.921875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.921875" style="1"/>
-    <col min="2" max="2" width="13.765625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.921875" style="1"/>
-    <col min="4" max="4" width="17.23046875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="13.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="17.21875" style="1" customWidth="1"/>
     <col min="5" max="5" width="22" style="1" customWidth="1"/>
-    <col min="6" max="7" width="23.3046875" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.921875" style="1"/>
+    <col min="6" max="7" width="23.33203125" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="49.85" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>5</v>
       </c>
@@ -946,7 +952,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -967,7 +973,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -990,7 +996,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="B4" s="3" t="s">
         <v>97</v>
@@ -1011,7 +1017,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -1020,7 +1026,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -1029,7 +1035,7 @@
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
     </row>
-    <row r="7" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -1038,7 +1044,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
     </row>
-    <row r="8" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -1047,7 +1053,7 @@
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
     </row>
-    <row r="9" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -1056,7 +1062,7 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
     </row>
-    <row r="10" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -1065,7 +1071,7 @@
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
     </row>
-    <row r="11" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -1074,7 +1080,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
     </row>
-    <row r="12" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -1083,7 +1089,7 @@
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
     </row>
-    <row r="13" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1092,7 +1098,7 @@
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
     </row>
-    <row r="14" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -1101,7 +1107,7 @@
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
     </row>
-    <row r="15" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -1118,120 +1124,119 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96C9021C-4823-4BF4-BE12-B962A68061DC}">
   <dimension ref="A1:AX20"/>
-  <sheetFormatPr defaultColWidth="8.921875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="8.921875" style="1"/>
-    <col min="3" max="3" width="11.23046875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.69140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.07421875" style="1" customWidth="1"/>
+    <col min="1" max="2" width="8.88671875" style="1"/>
+    <col min="3" max="3" width="11.21875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" style="1" customWidth="1"/>
     <col min="6" max="8" width="11" style="1" customWidth="1"/>
-    <col min="9" max="10" width="16.61328125" style="1" customWidth="1"/>
+    <col min="9" max="10" width="16.6640625" style="1" customWidth="1"/>
     <col min="11" max="14" width="21" style="1" customWidth="1"/>
-    <col min="15" max="15" width="13.765625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="19.3828125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="12.69140625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="13.77734375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="19.33203125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="12.6640625" style="1" customWidth="1"/>
     <col min="18" max="18" width="20" style="1" customWidth="1"/>
-    <col min="19" max="22" width="12.07421875" style="1" customWidth="1"/>
-    <col min="23" max="23" width="12.07421875" style="16" customWidth="1"/>
-    <col min="24" max="25" width="12.07421875" style="1" customWidth="1"/>
-    <col min="26" max="26" width="15.3828125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="20.23046875" style="1" customWidth="1"/>
-    <col min="28" max="28" width="16.61328125" style="1" customWidth="1"/>
-    <col min="29" max="29" width="17.23046875" style="1" customWidth="1"/>
-    <col min="30" max="30" width="11.07421875" style="1" customWidth="1"/>
-    <col min="31" max="31" width="12.69140625" style="1" customWidth="1"/>
-    <col min="32" max="32" width="12.61328125" style="1" customWidth="1"/>
-    <col min="33" max="33" width="12.07421875" style="1" customWidth="1"/>
-    <col min="34" max="34" width="12.3828125" style="1" customWidth="1"/>
+    <col min="19" max="22" width="12.109375" style="1" customWidth="1"/>
+    <col min="23" max="23" width="12.109375" style="16" customWidth="1"/>
+    <col min="24" max="25" width="12.109375" style="1" customWidth="1"/>
+    <col min="26" max="26" width="15.33203125" style="1" customWidth="1"/>
+    <col min="27" max="27" width="20.21875" style="1" customWidth="1"/>
+    <col min="28" max="28" width="16.6640625" style="1" customWidth="1"/>
+    <col min="29" max="29" width="17.21875" style="1" customWidth="1"/>
+    <col min="30" max="30" width="11.109375" style="1" customWidth="1"/>
+    <col min="31" max="32" width="12.6640625" style="1" customWidth="1"/>
+    <col min="33" max="33" width="12.109375" style="1" customWidth="1"/>
+    <col min="34" max="34" width="12.33203125" style="1" customWidth="1"/>
     <col min="35" max="35" width="14" style="1" customWidth="1"/>
-    <col min="36" max="36" width="12.3046875" style="1" customWidth="1"/>
-    <col min="37" max="37" width="12.765625" style="1" customWidth="1"/>
-    <col min="38" max="38" width="21.921875" style="1" customWidth="1"/>
-    <col min="39" max="39" width="19.23046875" style="1" customWidth="1"/>
-    <col min="40" max="40" width="15.765625" style="1" customWidth="1"/>
-    <col min="41" max="41" width="24.765625" style="1" customWidth="1"/>
-    <col min="42" max="44" width="15.69140625" style="1" customWidth="1"/>
-    <col min="45" max="45" width="14.69140625" style="1" customWidth="1"/>
-    <col min="46" max="46" width="17.921875" style="1" customWidth="1"/>
+    <col min="36" max="36" width="12.33203125" style="1" customWidth="1"/>
+    <col min="37" max="37" width="12.77734375" style="1" customWidth="1"/>
+    <col min="38" max="38" width="21.88671875" style="1" customWidth="1"/>
+    <col min="39" max="39" width="19.21875" style="1" customWidth="1"/>
+    <col min="40" max="40" width="15.77734375" style="1" customWidth="1"/>
+    <col min="41" max="41" width="24.77734375" style="1" customWidth="1"/>
+    <col min="42" max="44" width="15.6640625" style="1" customWidth="1"/>
+    <col min="45" max="45" width="14.6640625" style="1" customWidth="1"/>
+    <col min="46" max="46" width="17.88671875" style="1" customWidth="1"/>
     <col min="47" max="47" width="18" style="1" customWidth="1"/>
-    <col min="48" max="48" width="12.69140625" style="1" customWidth="1"/>
-    <col min="49" max="49" width="19.921875" style="1" customWidth="1"/>
-    <col min="50" max="50" width="26.765625" style="1" customWidth="1"/>
-    <col min="51" max="16384" width="8.921875" style="1"/>
+    <col min="48" max="48" width="12.6640625" style="1" customWidth="1"/>
+    <col min="49" max="49" width="19.88671875" style="1" customWidth="1"/>
+    <col min="50" max="50" width="26.77734375" style="1" customWidth="1"/>
+    <col min="51" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" ht="31.85" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:50" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23" t="s">
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
-      <c r="AA1" s="23" t="s">
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
+      <c r="R1" s="25"/>
+      <c r="S1" s="25"/>
+      <c r="T1" s="25"/>
+      <c r="U1" s="25"/>
+      <c r="V1" s="25"/>
+      <c r="W1" s="25"/>
+      <c r="X1" s="25"/>
+      <c r="Y1" s="25"/>
+      <c r="Z1" s="25"/>
+      <c r="AA1" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="AB1" s="23"/>
-      <c r="AC1" s="23"/>
-      <c r="AD1" s="23" t="s">
+      <c r="AB1" s="25"/>
+      <c r="AC1" s="25"/>
+      <c r="AD1" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="AE1" s="23"/>
-      <c r="AF1" s="23"/>
-      <c r="AG1" s="23"/>
-      <c r="AH1" s="23"/>
-      <c r="AI1" s="23"/>
-      <c r="AJ1" s="23"/>
-      <c r="AK1" s="23"/>
-      <c r="AL1" s="23"/>
-      <c r="AM1" s="23" t="s">
+      <c r="AE1" s="25"/>
+      <c r="AF1" s="25"/>
+      <c r="AG1" s="25"/>
+      <c r="AH1" s="25"/>
+      <c r="AI1" s="25"/>
+      <c r="AJ1" s="25"/>
+      <c r="AK1" s="25"/>
+      <c r="AL1" s="25"/>
+      <c r="AM1" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="AN1" s="23"/>
-      <c r="AO1" s="23" t="s">
+      <c r="AN1" s="25"/>
+      <c r="AO1" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AP1" s="23"/>
-      <c r="AQ1" s="23"/>
-      <c r="AR1" s="23"/>
-      <c r="AS1" s="23"/>
-      <c r="AT1" s="23" t="s">
+      <c r="AP1" s="25"/>
+      <c r="AQ1" s="25"/>
+      <c r="AR1" s="25"/>
+      <c r="AS1" s="25"/>
+      <c r="AT1" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="AU1" s="23"/>
-      <c r="AV1" s="23" t="s">
+      <c r="AU1" s="25"/>
+      <c r="AV1" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="AW1" s="23"/>
-      <c r="AX1" s="23"/>
-    </row>
-    <row r="2" spans="1:50" ht="49.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="25"/>
+      <c r="AW1" s="25"/>
+      <c r="AX1" s="25"/>
+    </row>
+    <row r="2" spans="1:50" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="27"/>
       <c r="B2" s="12" t="s">
         <v>33</v>
       </c>
@@ -1380,7 +1385,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -1452,7 +1457,7 @@
       <c r="AW3" s="10"/>
       <c r="AX3" s="10"/>
     </row>
-    <row r="4" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -1504,7 +1509,7 @@
       <c r="AW4" s="10"/>
       <c r="AX4" s="10"/>
     </row>
-    <row r="5" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -1556,7 +1561,7 @@
       <c r="AW5" s="10"/>
       <c r="AX5" s="10"/>
     </row>
-    <row r="6" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -1608,7 +1613,7 @@
       <c r="AW6" s="10"/>
       <c r="AX6" s="10"/>
     </row>
-    <row r="7" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -1660,7 +1665,7 @@
       <c r="AW7" s="10"/>
       <c r="AX7" s="10"/>
     </row>
-    <row r="8" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -1712,7 +1717,7 @@
       <c r="AW8" s="10"/>
       <c r="AX8" s="10"/>
     </row>
-    <row r="9" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -1764,7 +1769,7 @@
       <c r="AW9" s="10"/>
       <c r="AX9" s="10"/>
     </row>
-    <row r="10" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -1816,7 +1821,7 @@
       <c r="AW10" s="10"/>
       <c r="AX10" s="10"/>
     </row>
-    <row r="11" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -1868,7 +1873,7 @@
       <c r="AW11" s="10"/>
       <c r="AX11" s="10"/>
     </row>
-    <row r="12" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -1920,7 +1925,7 @@
       <c r="AW12" s="10"/>
       <c r="AX12" s="10"/>
     </row>
-    <row r="13" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -1972,7 +1977,7 @@
       <c r="AW13" s="10"/>
       <c r="AX13" s="10"/>
     </row>
-    <row r="14" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -2024,7 +2029,7 @@
       <c r="AW14" s="10"/>
       <c r="AX14" s="10"/>
     </row>
-    <row r="15" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -2076,7 +2081,7 @@
       <c r="AW15" s="10"/>
       <c r="AX15" s="10"/>
     </row>
-    <row r="16" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -2128,7 +2133,7 @@
       <c r="AW16" s="10"/>
       <c r="AX16" s="10"/>
     </row>
-    <row r="17" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -2180,7 +2185,7 @@
       <c r="AW17" s="10"/>
       <c r="AX17" s="10"/>
     </row>
-    <row r="18" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -2232,7 +2237,7 @@
       <c r="AW18" s="10"/>
       <c r="AX18" s="10"/>
     </row>
-    <row r="19" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -2284,7 +2289,7 @@
       <c r="AW19" s="10"/>
       <c r="AX19" s="10"/>
     </row>
-    <row r="20" spans="1:50" ht="100.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:50" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -2354,27 +2359,27 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S101"/>
-  <sheetFormatPr defaultColWidth="8.921875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:S100"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.69140625" style="1" customWidth="1"/>
-    <col min="2" max="3" width="18.3046875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.3828125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" style="1" customWidth="1"/>
+    <col min="2" max="3" width="18.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="16" style="1" customWidth="1"/>
-    <col min="6" max="7" width="16.765625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="22.07421875" style="1" customWidth="1"/>
-    <col min="9" max="12" width="16.07421875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="13.23046875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="17.765625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="11.3828125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="9.3828125" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.69140625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="21.69140625" style="1" customWidth="1"/>
-    <col min="19" max="19" width="14.07421875" style="1" customWidth="1"/>
-    <col min="20" max="16384" width="8.921875" style="1"/>
+    <col min="6" max="7" width="16.77734375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="22.109375" style="1" customWidth="1"/>
+    <col min="9" max="12" width="16.109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13.21875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="17.77734375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="11.33203125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.6640625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="21.6640625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="14.109375" style="1" customWidth="1"/>
+    <col min="20" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="64.849999999999994" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:19" ht="64.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>5</v>
       </c>
@@ -2433,7 +2438,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2493,11 +2498,13 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="8"/>
+      <c r="B3" s="8" t="s">
+        <v>98</v>
+      </c>
       <c r="C3" s="8" t="s">
         <v>97</v>
       </c>
@@ -2526,24 +2533,37 @@
         <v>100</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
-      <c r="Q3" s="18"/>
-      <c r="R3" s="18"/>
+        <v>99</v>
+      </c>
+      <c r="M3" s="18">
+        <v>0.46614</v>
+      </c>
+      <c r="N3" s="18">
+        <v>0.23693</v>
+      </c>
+      <c r="O3" s="18">
+        <v>0.5343</v>
+      </c>
+      <c r="P3" s="18">
+        <v>0.44085999999999997</v>
+      </c>
+      <c r="Q3" s="18">
+        <f t="shared" ref="Q3:Q8" si="0">2*(O3*P3)/(O3+P3)</f>
+        <v>0.48310328151277737</v>
+      </c>
+      <c r="R3" s="18">
+        <v>0.6</v>
+      </c>
       <c r="S3" s="19">
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>97</v>
@@ -2558,7 +2578,7 @@
         <v>36</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>37</v>
+        <v>102</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>25</v>
@@ -2573,37 +2593,37 @@
         <v>100</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>99</v>
+        <v>26</v>
       </c>
       <c r="M4" s="18">
-        <v>0.46614</v>
+        <v>0.53337000000000001</v>
       </c>
       <c r="N4" s="18">
-        <v>0.23693</v>
+        <v>0.29136000000000001</v>
       </c>
       <c r="O4" s="18">
-        <v>0.5343</v>
+        <v>0.57379999999999998</v>
       </c>
       <c r="P4" s="18">
-        <v>0.44085999999999997</v>
+        <v>0.54252</v>
       </c>
       <c r="Q4" s="18">
-        <f t="shared" ref="Q4:Q8" si="0">2*(O4*P4)/(O4+P4)</f>
-        <v>0.48310328151277737</v>
+        <f t="shared" si="0"/>
+        <v>0.55772175720223593</v>
       </c>
       <c r="R4" s="18">
-        <v>0.6</v>
+        <v>1.7</v>
       </c>
       <c r="S4" s="19">
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>97</v>
@@ -2618,7 +2638,7 @@
         <v>36</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>25</v>
@@ -2636,34 +2656,34 @@
         <v>26</v>
       </c>
       <c r="M5" s="18">
-        <v>0.53337000000000001</v>
+        <v>0.56028999999999995</v>
       </c>
       <c r="N5" s="18">
-        <v>0.29136000000000001</v>
+        <v>0.31753999999999999</v>
       </c>
       <c r="O5" s="18">
-        <v>0.57379999999999998</v>
+        <v>0.59638999999999998</v>
       </c>
       <c r="P5" s="18">
-        <v>0.54252</v>
+        <v>0.55254999999999999</v>
       </c>
       <c r="Q5" s="18">
         <f t="shared" si="0"/>
-        <v>0.55772175720223593</v>
+        <v>0.57363360053614632</v>
       </c>
       <c r="R5" s="18">
-        <v>1.7</v>
+        <v>3.2</v>
       </c>
       <c r="S5" s="19">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>97</v>
@@ -2678,7 +2698,7 @@
         <v>36</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>25</v>
@@ -2696,34 +2716,34 @@
         <v>26</v>
       </c>
       <c r="M6" s="18">
-        <v>0.56028999999999995</v>
+        <v>0.57698000000000005</v>
       </c>
       <c r="N6" s="18">
-        <v>0.31753999999999999</v>
+        <v>0.33145000000000002</v>
       </c>
       <c r="O6" s="18">
-        <v>0.59638999999999998</v>
+        <v>0.628</v>
       </c>
       <c r="P6" s="18">
-        <v>0.55254999999999999</v>
+        <v>0.57833000000000001</v>
       </c>
       <c r="Q6" s="18">
         <f t="shared" si="0"/>
-        <v>0.57363360053614632</v>
+        <v>0.60214243200450968</v>
       </c>
       <c r="R6" s="18">
-        <v>3.2</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="S6" s="19">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>5</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>105</v>
+        <v>6</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>108</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>97</v>
@@ -2738,7 +2758,7 @@
         <v>36</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>25</v>
@@ -2756,34 +2776,34 @@
         <v>26</v>
       </c>
       <c r="M7" s="18">
-        <v>0.57698000000000005</v>
+        <v>0.59257000000000004</v>
       </c>
       <c r="N7" s="18">
-        <v>0.33145000000000002</v>
+        <v>0.35102</v>
       </c>
       <c r="O7" s="18">
-        <v>0.628</v>
+        <v>0.62219999999999998</v>
       </c>
       <c r="P7" s="18">
-        <v>0.57833000000000001</v>
+        <v>0.58816000000000002</v>
       </c>
       <c r="Q7" s="18">
         <f t="shared" si="0"/>
-        <v>0.60214243200450968</v>
+        <v>0.6047013318351564</v>
       </c>
       <c r="R7" s="18">
-        <v>4.9000000000000004</v>
+        <v>7.8</v>
       </c>
       <c r="S7" s="19">
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>6</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>107</v>
+        <v>7</v>
+      </c>
+      <c r="B8" s="24">
+        <v>46059</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>97</v>
@@ -2798,7 +2818,7 @@
         <v>36</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>108</v>
+        <v>37</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>25</v>
@@ -2816,27 +2836,29 @@
         <v>26</v>
       </c>
       <c r="M8" s="18">
-        <v>0.59257000000000004</v>
+        <v>0.49164999999999998</v>
       </c>
       <c r="N8" s="18">
-        <v>0.35102</v>
+        <v>0.25875999999999999</v>
       </c>
       <c r="O8" s="18">
-        <v>0.62219999999999998</v>
+        <v>0.52237</v>
       </c>
       <c r="P8" s="18">
-        <v>0.58816000000000002</v>
+        <v>0.50277000000000005</v>
       </c>
       <c r="Q8" s="18">
         <f t="shared" si="0"/>
-        <v>0.6047013318351564</v>
-      </c>
-      <c r="R8" s="18"/>
+        <v>0.51238263046998467</v>
+      </c>
+      <c r="R8" s="18">
+        <v>1</v>
+      </c>
       <c r="S8" s="19">
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -2857,7 +2879,7 @@
       <c r="R9" s="18"/>
       <c r="S9" s="19"/>
     </row>
-    <row r="10" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -2878,7 +2900,7 @@
       <c r="R10" s="18"/>
       <c r="S10" s="19"/>
     </row>
-    <row r="11" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -2899,7 +2921,7 @@
       <c r="R11" s="18"/>
       <c r="S11" s="19"/>
     </row>
-    <row r="12" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -2920,7 +2942,7 @@
       <c r="R12" s="18"/>
       <c r="S12" s="19"/>
     </row>
-    <row r="13" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -2941,7 +2963,7 @@
       <c r="R13" s="18"/>
       <c r="S13" s="19"/>
     </row>
-    <row r="14" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -2962,7 +2984,7 @@
       <c r="R14" s="18"/>
       <c r="S14" s="19"/>
     </row>
-    <row r="15" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -2983,7 +3005,7 @@
       <c r="R15" s="18"/>
       <c r="S15" s="19"/>
     </row>
-    <row r="16" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -3004,7 +3026,7 @@
       <c r="R16" s="18"/>
       <c r="S16" s="19"/>
     </row>
-    <row r="17" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -3025,7 +3047,7 @@
       <c r="R17" s="18"/>
       <c r="S17" s="19"/>
     </row>
-    <row r="18" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -3046,7 +3068,7 @@
       <c r="R18" s="18"/>
       <c r="S18" s="19"/>
     </row>
-    <row r="19" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -3067,7 +3089,7 @@
       <c r="R19" s="18"/>
       <c r="S19" s="19"/>
     </row>
-    <row r="20" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -3088,7 +3110,7 @@
       <c r="R20" s="18"/>
       <c r="S20" s="19"/>
     </row>
-    <row r="21" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -3109,7 +3131,7 @@
       <c r="R21" s="18"/>
       <c r="S21" s="19"/>
     </row>
-    <row r="22" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -3130,7 +3152,7 @@
       <c r="R22" s="18"/>
       <c r="S22" s="19"/>
     </row>
-    <row r="23" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -3151,7 +3173,7 @@
       <c r="R23" s="18"/>
       <c r="S23" s="19"/>
     </row>
-    <row r="24" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -3172,7 +3194,7 @@
       <c r="R24" s="18"/>
       <c r="S24" s="19"/>
     </row>
-    <row r="25" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -3193,7 +3215,7 @@
       <c r="R25" s="18"/>
       <c r="S25" s="19"/>
     </row>
-    <row r="26" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -3214,7 +3236,7 @@
       <c r="R26" s="18"/>
       <c r="S26" s="19"/>
     </row>
-    <row r="27" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -3235,7 +3257,7 @@
       <c r="R27" s="18"/>
       <c r="S27" s="19"/>
     </row>
-    <row r="28" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -3256,7 +3278,7 @@
       <c r="R28" s="18"/>
       <c r="S28" s="19"/>
     </row>
-    <row r="29" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -3277,7 +3299,7 @@
       <c r="R29" s="18"/>
       <c r="S29" s="19"/>
     </row>
-    <row r="30" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
@@ -3298,7 +3320,7 @@
       <c r="R30" s="18"/>
       <c r="S30" s="19"/>
     </row>
-    <row r="31" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
       <c r="B31" s="8"/>
       <c r="C31" s="8"/>
@@ -3319,7 +3341,7 @@
       <c r="R31" s="18"/>
       <c r="S31" s="19"/>
     </row>
-    <row r="32" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
@@ -3340,7 +3362,7 @@
       <c r="R32" s="18"/>
       <c r="S32" s="19"/>
     </row>
-    <row r="33" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
@@ -3361,7 +3383,7 @@
       <c r="R33" s="18"/>
       <c r="S33" s="19"/>
     </row>
-    <row r="34" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -3382,7 +3404,7 @@
       <c r="R34" s="18"/>
       <c r="S34" s="19"/>
     </row>
-    <row r="35" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
@@ -3403,7 +3425,7 @@
       <c r="R35" s="18"/>
       <c r="S35" s="19"/>
     </row>
-    <row r="36" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -3424,7 +3446,7 @@
       <c r="R36" s="18"/>
       <c r="S36" s="19"/>
     </row>
-    <row r="37" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -3445,7 +3467,7 @@
       <c r="R37" s="18"/>
       <c r="S37" s="19"/>
     </row>
-    <row r="38" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
       <c r="B38" s="8"/>
       <c r="C38" s="8"/>
@@ -3466,7 +3488,7 @@
       <c r="R38" s="18"/>
       <c r="S38" s="19"/>
     </row>
-    <row r="39" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
@@ -3487,7 +3509,7 @@
       <c r="R39" s="18"/>
       <c r="S39" s="19"/>
     </row>
-    <row r="40" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
@@ -3508,7 +3530,7 @@
       <c r="R40" s="18"/>
       <c r="S40" s="19"/>
     </row>
-    <row r="41" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
@@ -3529,7 +3551,7 @@
       <c r="R41" s="18"/>
       <c r="S41" s="19"/>
     </row>
-    <row r="42" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
@@ -3550,7 +3572,7 @@
       <c r="R42" s="18"/>
       <c r="S42" s="19"/>
     </row>
-    <row r="43" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
@@ -3571,7 +3593,7 @@
       <c r="R43" s="18"/>
       <c r="S43" s="19"/>
     </row>
-    <row r="44" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -3592,7 +3614,7 @@
       <c r="R44" s="18"/>
       <c r="S44" s="19"/>
     </row>
-    <row r="45" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -3613,7 +3635,7 @@
       <c r="R45" s="18"/>
       <c r="S45" s="19"/>
     </row>
-    <row r="46" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -3634,7 +3656,7 @@
       <c r="R46" s="18"/>
       <c r="S46" s="19"/>
     </row>
-    <row r="47" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
@@ -3655,7 +3677,7 @@
       <c r="R47" s="18"/>
       <c r="S47" s="19"/>
     </row>
-    <row r="48" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
@@ -3676,7 +3698,7 @@
       <c r="R48" s="18"/>
       <c r="S48" s="19"/>
     </row>
-    <row r="49" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
@@ -3697,7 +3719,7 @@
       <c r="R49" s="18"/>
       <c r="S49" s="19"/>
     </row>
-    <row r="50" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
@@ -3718,7 +3740,7 @@
       <c r="R50" s="18"/>
       <c r="S50" s="19"/>
     </row>
-    <row r="51" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="8"/>
       <c r="C51" s="8"/>
@@ -3739,7 +3761,7 @@
       <c r="R51" s="18"/>
       <c r="S51" s="19"/>
     </row>
-    <row r="52" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
@@ -3760,7 +3782,7 @@
       <c r="R52" s="18"/>
       <c r="S52" s="19"/>
     </row>
-    <row r="53" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="8"/>
       <c r="C53" s="8"/>
@@ -3781,7 +3803,7 @@
       <c r="R53" s="18"/>
       <c r="S53" s="19"/>
     </row>
-    <row r="54" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
       <c r="B54" s="8"/>
       <c r="C54" s="8"/>
@@ -3802,7 +3824,7 @@
       <c r="R54" s="18"/>
       <c r="S54" s="19"/>
     </row>
-    <row r="55" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2"/>
       <c r="B55" s="8"/>
       <c r="C55" s="8"/>
@@ -3823,7 +3845,7 @@
       <c r="R55" s="18"/>
       <c r="S55" s="19"/>
     </row>
-    <row r="56" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2"/>
       <c r="B56" s="8"/>
       <c r="C56" s="8"/>
@@ -3844,7 +3866,7 @@
       <c r="R56" s="18"/>
       <c r="S56" s="19"/>
     </row>
-    <row r="57" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2"/>
       <c r="B57" s="8"/>
       <c r="C57" s="8"/>
@@ -3865,7 +3887,7 @@
       <c r="R57" s="18"/>
       <c r="S57" s="19"/>
     </row>
-    <row r="58" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2"/>
       <c r="B58" s="8"/>
       <c r="C58" s="8"/>
@@ -3886,7 +3908,7 @@
       <c r="R58" s="18"/>
       <c r="S58" s="19"/>
     </row>
-    <row r="59" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
       <c r="B59" s="8"/>
       <c r="C59" s="8"/>
@@ -3907,7 +3929,7 @@
       <c r="R59" s="18"/>
       <c r="S59" s="19"/>
     </row>
-    <row r="60" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2"/>
       <c r="B60" s="8"/>
       <c r="C60" s="8"/>
@@ -3928,7 +3950,7 @@
       <c r="R60" s="18"/>
       <c r="S60" s="19"/>
     </row>
-    <row r="61" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2"/>
       <c r="B61" s="8"/>
       <c r="C61" s="8"/>
@@ -3949,7 +3971,7 @@
       <c r="R61" s="18"/>
       <c r="S61" s="19"/>
     </row>
-    <row r="62" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2"/>
       <c r="B62" s="8"/>
       <c r="C62" s="8"/>
@@ -3970,7 +3992,7 @@
       <c r="R62" s="18"/>
       <c r="S62" s="19"/>
     </row>
-    <row r="63" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2"/>
       <c r="B63" s="8"/>
       <c r="C63" s="8"/>
@@ -3991,7 +4013,7 @@
       <c r="R63" s="18"/>
       <c r="S63" s="19"/>
     </row>
-    <row r="64" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2"/>
       <c r="B64" s="8"/>
       <c r="C64" s="8"/>
@@ -4012,7 +4034,7 @@
       <c r="R64" s="18"/>
       <c r="S64" s="19"/>
     </row>
-    <row r="65" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2"/>
       <c r="B65" s="8"/>
       <c r="C65" s="8"/>
@@ -4033,7 +4055,7 @@
       <c r="R65" s="18"/>
       <c r="S65" s="19"/>
     </row>
-    <row r="66" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2"/>
       <c r="B66" s="8"/>
       <c r="C66" s="8"/>
@@ -4054,7 +4076,7 @@
       <c r="R66" s="18"/>
       <c r="S66" s="19"/>
     </row>
-    <row r="67" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2"/>
       <c r="B67" s="8"/>
       <c r="C67" s="8"/>
@@ -4075,7 +4097,7 @@
       <c r="R67" s="18"/>
       <c r="S67" s="19"/>
     </row>
-    <row r="68" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
       <c r="B68" s="8"/>
       <c r="C68" s="8"/>
@@ -4096,7 +4118,7 @@
       <c r="R68" s="18"/>
       <c r="S68" s="19"/>
     </row>
-    <row r="69" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2"/>
       <c r="B69" s="8"/>
       <c r="C69" s="8"/>
@@ -4117,7 +4139,7 @@
       <c r="R69" s="18"/>
       <c r="S69" s="19"/>
     </row>
-    <row r="70" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2"/>
       <c r="B70" s="8"/>
       <c r="C70" s="8"/>
@@ -4138,7 +4160,7 @@
       <c r="R70" s="18"/>
       <c r="S70" s="19"/>
     </row>
-    <row r="71" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2"/>
       <c r="B71" s="8"/>
       <c r="C71" s="8"/>
@@ -4159,7 +4181,7 @@
       <c r="R71" s="18"/>
       <c r="S71" s="19"/>
     </row>
-    <row r="72" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2"/>
       <c r="B72" s="8"/>
       <c r="C72" s="8"/>
@@ -4180,7 +4202,7 @@
       <c r="R72" s="18"/>
       <c r="S72" s="19"/>
     </row>
-    <row r="73" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2"/>
       <c r="B73" s="8"/>
       <c r="C73" s="8"/>
@@ -4201,7 +4223,7 @@
       <c r="R73" s="18"/>
       <c r="S73" s="19"/>
     </row>
-    <row r="74" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2"/>
       <c r="B74" s="8"/>
       <c r="C74" s="8"/>
@@ -4222,7 +4244,7 @@
       <c r="R74" s="18"/>
       <c r="S74" s="19"/>
     </row>
-    <row r="75" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="2"/>
       <c r="B75" s="8"/>
       <c r="C75" s="8"/>
@@ -4243,7 +4265,7 @@
       <c r="R75" s="18"/>
       <c r="S75" s="19"/>
     </row>
-    <row r="76" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="2"/>
       <c r="B76" s="8"/>
       <c r="C76" s="8"/>
@@ -4264,7 +4286,7 @@
       <c r="R76" s="18"/>
       <c r="S76" s="19"/>
     </row>
-    <row r="77" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="2"/>
       <c r="B77" s="8"/>
       <c r="C77" s="8"/>
@@ -4285,7 +4307,7 @@
       <c r="R77" s="18"/>
       <c r="S77" s="19"/>
     </row>
-    <row r="78" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="2"/>
       <c r="B78" s="8"/>
       <c r="C78" s="8"/>
@@ -4306,7 +4328,7 @@
       <c r="R78" s="18"/>
       <c r="S78" s="19"/>
     </row>
-    <row r="79" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2"/>
       <c r="B79" s="8"/>
       <c r="C79" s="8"/>
@@ -4327,7 +4349,7 @@
       <c r="R79" s="18"/>
       <c r="S79" s="19"/>
     </row>
-    <row r="80" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="2"/>
       <c r="B80" s="8"/>
       <c r="C80" s="8"/>
@@ -4348,7 +4370,7 @@
       <c r="R80" s="18"/>
       <c r="S80" s="19"/>
     </row>
-    <row r="81" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2"/>
       <c r="B81" s="8"/>
       <c r="C81" s="8"/>
@@ -4369,7 +4391,7 @@
       <c r="R81" s="18"/>
       <c r="S81" s="19"/>
     </row>
-    <row r="82" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2"/>
       <c r="B82" s="8"/>
       <c r="C82" s="8"/>
@@ -4390,7 +4412,7 @@
       <c r="R82" s="18"/>
       <c r="S82" s="19"/>
     </row>
-    <row r="83" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2"/>
       <c r="B83" s="8"/>
       <c r="C83" s="8"/>
@@ -4411,7 +4433,7 @@
       <c r="R83" s="18"/>
       <c r="S83" s="19"/>
     </row>
-    <row r="84" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2"/>
       <c r="B84" s="8"/>
       <c r="C84" s="8"/>
@@ -4432,7 +4454,7 @@
       <c r="R84" s="18"/>
       <c r="S84" s="19"/>
     </row>
-    <row r="85" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2"/>
       <c r="B85" s="8"/>
       <c r="C85" s="8"/>
@@ -4453,7 +4475,7 @@
       <c r="R85" s="18"/>
       <c r="S85" s="19"/>
     </row>
-    <row r="86" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2"/>
       <c r="B86" s="8"/>
       <c r="C86" s="8"/>
@@ -4474,7 +4496,7 @@
       <c r="R86" s="18"/>
       <c r="S86" s="19"/>
     </row>
-    <row r="87" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2"/>
       <c r="B87" s="8"/>
       <c r="C87" s="8"/>
@@ -4495,7 +4517,7 @@
       <c r="R87" s="18"/>
       <c r="S87" s="19"/>
     </row>
-    <row r="88" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="2"/>
       <c r="B88" s="8"/>
       <c r="C88" s="8"/>
@@ -4516,7 +4538,7 @@
       <c r="R88" s="18"/>
       <c r="S88" s="19"/>
     </row>
-    <row r="89" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2"/>
       <c r="B89" s="8"/>
       <c r="C89" s="8"/>
@@ -4537,7 +4559,7 @@
       <c r="R89" s="18"/>
       <c r="S89" s="19"/>
     </row>
-    <row r="90" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2"/>
       <c r="B90" s="8"/>
       <c r="C90" s="8"/>
@@ -4558,7 +4580,7 @@
       <c r="R90" s="18"/>
       <c r="S90" s="19"/>
     </row>
-    <row r="91" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2"/>
       <c r="B91" s="8"/>
       <c r="C91" s="8"/>
@@ -4579,7 +4601,7 @@
       <c r="R91" s="18"/>
       <c r="S91" s="19"/>
     </row>
-    <row r="92" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2"/>
       <c r="B92" s="8"/>
       <c r="C92" s="8"/>
@@ -4600,7 +4622,7 @@
       <c r="R92" s="18"/>
       <c r="S92" s="19"/>
     </row>
-    <row r="93" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2"/>
       <c r="B93" s="8"/>
       <c r="C93" s="8"/>
@@ -4621,7 +4643,7 @@
       <c r="R93" s="18"/>
       <c r="S93" s="19"/>
     </row>
-    <row r="94" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2"/>
       <c r="B94" s="8"/>
       <c r="C94" s="8"/>
@@ -4642,7 +4664,7 @@
       <c r="R94" s="18"/>
       <c r="S94" s="19"/>
     </row>
-    <row r="95" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2"/>
       <c r="B95" s="8"/>
       <c r="C95" s="8"/>
@@ -4663,7 +4685,7 @@
       <c r="R95" s="18"/>
       <c r="S95" s="19"/>
     </row>
-    <row r="96" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2"/>
       <c r="B96" s="8"/>
       <c r="C96" s="8"/>
@@ -4684,7 +4706,7 @@
       <c r="R96" s="18"/>
       <c r="S96" s="19"/>
     </row>
-    <row r="97" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2"/>
       <c r="B97" s="8"/>
       <c r="C97" s="8"/>
@@ -4705,7 +4727,7 @@
       <c r="R97" s="18"/>
       <c r="S97" s="19"/>
     </row>
-    <row r="98" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2"/>
       <c r="B98" s="8"/>
       <c r="C98" s="8"/>
@@ -4726,7 +4748,7 @@
       <c r="R98" s="18"/>
       <c r="S98" s="19"/>
     </row>
-    <row r="99" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="2"/>
       <c r="B99" s="8"/>
       <c r="C99" s="8"/>
@@ -4747,7 +4769,7 @@
       <c r="R99" s="18"/>
       <c r="S99" s="19"/>
     </row>
-    <row r="100" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
       <c r="B100" s="8"/>
       <c r="C100" s="8"/>
@@ -4768,27 +4790,6 @@
       <c r="R100" s="18"/>
       <c r="S100" s="19"/>
     </row>
-    <row r="101" spans="1:19" ht="40.1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A101" s="2"/>
-      <c r="B101" s="8"/>
-      <c r="C101" s="8"/>
-      <c r="D101" s="8"/>
-      <c r="E101" s="9"/>
-      <c r="F101" s="9"/>
-      <c r="G101" s="9"/>
-      <c r="H101" s="9"/>
-      <c r="I101" s="9"/>
-      <c r="J101" s="9"/>
-      <c r="K101" s="9"/>
-      <c r="L101" s="9"/>
-      <c r="M101" s="18"/>
-      <c r="N101" s="18"/>
-      <c r="O101" s="18"/>
-      <c r="P101" s="18"/>
-      <c r="Q101" s="18"/>
-      <c r="R101" s="18"/>
-      <c r="S101" s="19"/>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="N1" r:id="rId1" xr:uid="{9B80FE5D-6B4B-4452-8753-71F3BE20CB96}"/>

</xml_diff>

<commit_message>
added train results 8 to 12, for model version 9
</commit_message>
<xml_diff>
--- a/work.xlsx
+++ b/work.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\iman_heydardoost\research_papers\dental_paper_1\Dental-XRay-YOLO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A513935-B642-478A-8CDA-3B4BD7AA3C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F7D218-9DAA-402A-8E04-F6528BAC2CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="660" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="116">
   <si>
     <t>number of models in series</t>
   </si>
@@ -383,6 +383,27 @@
   </si>
   <si>
     <t>21/2/2026 rerun:28/5/2026</t>
+  </si>
+  <si>
+    <t>YOLOv9</t>
+  </si>
+  <si>
+    <t>tiny</t>
+  </si>
+  <si>
+    <t>compact</t>
+  </si>
+  <si>
+    <t>extended</t>
+  </si>
+  <si>
+    <t>YOLOv10</t>
+  </si>
+  <si>
+    <t>balanced</t>
+  </si>
+  <si>
+    <t>extra large</t>
   </si>
 </sst>
 </file>
@@ -2362,17 +2383,17 @@
   <dimension ref="A1:S100"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.109375" style="1" customWidth="1"/>
     <col min="2" max="3" width="18.33203125" style="1" customWidth="1"/>
     <col min="4" max="4" width="16.33203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="16" style="1" customWidth="1"/>
     <col min="6" max="7" width="16.77734375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="22.109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" style="1" customWidth="1"/>
     <col min="9" max="12" width="16.109375" style="1" customWidth="1"/>
     <col min="13" max="13" width="13.21875" style="1" customWidth="1"/>
     <col min="14" max="14" width="17.77734375" style="1" customWidth="1"/>
     <col min="15" max="15" width="11.33203125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12" style="1" customWidth="1"/>
     <col min="17" max="17" width="12.6640625" style="1" customWidth="1"/>
     <col min="18" max="18" width="21.6640625" style="1" customWidth="1"/>
     <col min="19" max="19" width="14.109375" style="1" customWidth="1"/>
@@ -2548,7 +2569,7 @@
         <v>0.44085999999999997</v>
       </c>
       <c r="Q3" s="18">
-        <f t="shared" ref="Q3:Q8" si="0">2*(O3*P3)/(O3+P3)</f>
+        <f t="shared" ref="Q3:Q13" si="0">2*(O3*P3)/(O3+P3)</f>
         <v>0.48310328151277737</v>
       </c>
       <c r="R3" s="18">
@@ -2859,123 +2880,342 @@
       </c>
     </row>
     <row r="9" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="18"/>
-      <c r="N9" s="18"/>
-      <c r="O9" s="18"/>
-      <c r="P9" s="18"/>
-      <c r="Q9" s="18"/>
-      <c r="R9" s="18"/>
-      <c r="S9" s="19"/>
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="24">
+        <v>46209</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D9" s="8">
+        <v>1</v>
+      </c>
+      <c r="E9" s="9">
+        <v>1</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I9" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J9" s="9">
+        <v>16</v>
+      </c>
+      <c r="K9" s="9">
+        <v>100</v>
+      </c>
+      <c r="L9" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" s="18">
+        <v>0.48100999999999999</v>
+      </c>
+      <c r="N9" s="18">
+        <v>0.24918999999999999</v>
+      </c>
+      <c r="O9" s="18">
+        <v>0.50044999999999995</v>
+      </c>
+      <c r="P9" s="18">
+        <v>0.51924000000000003</v>
+      </c>
+      <c r="Q9" s="18">
+        <f t="shared" si="0"/>
+        <v>0.50967187674685444</v>
+      </c>
+      <c r="R9" s="18">
+        <v>0.6</v>
+      </c>
+      <c r="S9" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="10" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="18"/>
-      <c r="N10" s="18"/>
-      <c r="O10" s="18"/>
-      <c r="P10" s="18"/>
-      <c r="Q10" s="18"/>
-      <c r="R10" s="18"/>
-      <c r="S10" s="19"/>
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="24">
+        <v>46209</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D10" s="8">
+        <v>1</v>
+      </c>
+      <c r="E10" s="9">
+        <v>1</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J10" s="9">
+        <v>16</v>
+      </c>
+      <c r="K10" s="9">
+        <v>100</v>
+      </c>
+      <c r="L10" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" s="18">
+        <v>0.52519000000000005</v>
+      </c>
+      <c r="N10" s="18">
+        <v>0.28211000000000003</v>
+      </c>
+      <c r="O10" s="18">
+        <v>0.54549999999999998</v>
+      </c>
+      <c r="P10" s="18">
+        <v>0.54286000000000001</v>
+      </c>
+      <c r="Q10" s="18">
+        <f t="shared" si="0"/>
+        <v>0.54417679811826969</v>
+      </c>
+      <c r="R10" s="18">
+        <v>0.7</v>
+      </c>
+      <c r="S10" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="11" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="18"/>
-      <c r="N11" s="18"/>
-      <c r="O11" s="18"/>
-      <c r="P11" s="18"/>
-      <c r="Q11" s="18"/>
-      <c r="R11" s="18"/>
-      <c r="S11" s="19"/>
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="24">
+        <v>46240</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D11" s="8">
+        <v>1</v>
+      </c>
+      <c r="E11" s="9">
+        <v>1</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I11" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J11" s="9">
+        <v>16</v>
+      </c>
+      <c r="K11" s="9">
+        <v>100</v>
+      </c>
+      <c r="L11" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M11" s="18">
+        <v>0.54954999999999998</v>
+      </c>
+      <c r="N11" s="18">
+        <v>0.30653000000000002</v>
+      </c>
+      <c r="O11" s="18">
+        <v>0.57633000000000001</v>
+      </c>
+      <c r="P11" s="18">
+        <v>0.56303999999999998</v>
+      </c>
+      <c r="Q11" s="18">
+        <f>2*(O11*P11)/(O11+P11)</f>
+        <v>0.56960749045525161</v>
+      </c>
+      <c r="R11" s="18">
+        <v>1.3</v>
+      </c>
+      <c r="S11" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="12" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="18"/>
-      <c r="N12" s="18"/>
-      <c r="O12" s="18"/>
-      <c r="P12" s="18"/>
-      <c r="Q12" s="18"/>
-      <c r="R12" s="18"/>
-      <c r="S12" s="19"/>
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="24">
+        <v>46240</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="8">
+        <v>1</v>
+      </c>
+      <c r="E12" s="9">
+        <v>1</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I12" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J12" s="9">
+        <v>16</v>
+      </c>
+      <c r="K12" s="9">
+        <v>100</v>
+      </c>
+      <c r="L12" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M12" s="18">
+        <v>0.56130000000000002</v>
+      </c>
+      <c r="N12" s="18">
+        <v>0.31719999999999998</v>
+      </c>
+      <c r="O12" s="18">
+        <v>0.59931999999999996</v>
+      </c>
+      <c r="P12" s="18">
+        <v>0.56494999999999995</v>
+      </c>
+      <c r="Q12" s="18">
+        <f t="shared" si="0"/>
+        <v>0.58162768773566265</v>
+      </c>
+      <c r="R12" s="18">
+        <v>1.6</v>
+      </c>
+      <c r="S12" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="13" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="18"/>
-      <c r="N13" s="18"/>
-      <c r="O13" s="18"/>
-      <c r="P13" s="18"/>
-      <c r="Q13" s="18"/>
-      <c r="R13" s="18"/>
-      <c r="S13" s="19"/>
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="24">
+        <v>46271</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D13" s="8">
+        <v>1</v>
+      </c>
+      <c r="E13" s="9">
+        <v>1</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I13" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J13" s="9">
+        <v>16</v>
+      </c>
+      <c r="K13" s="9">
+        <v>100</v>
+      </c>
+      <c r="L13" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M13" s="18">
+        <v>0.59708000000000006</v>
+      </c>
+      <c r="N13" s="18">
+        <v>0.34964000000000001</v>
+      </c>
+      <c r="O13" s="18">
+        <v>0.65808</v>
+      </c>
+      <c r="P13" s="18">
+        <v>0.58526999999999996</v>
+      </c>
+      <c r="Q13" s="18">
+        <f t="shared" si="0"/>
+        <v>0.61954314006514655</v>
+      </c>
+      <c r="R13" s="18">
+        <v>3.7</v>
+      </c>
+      <c r="S13" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="14" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="24">
+        <v>46301</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D14" s="8">
+        <v>1</v>
+      </c>
+      <c r="E14" s="9">
+        <v>1</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I14" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J14" s="9">
+        <v>16</v>
+      </c>
+      <c r="K14" s="9">
+        <v>100</v>
+      </c>
+      <c r="L14" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M14" s="18"/>
       <c r="N14" s="18"/>
       <c r="O14" s="18"/>
@@ -2985,18 +3225,40 @@
       <c r="S14" s="19"/>
     </row>
     <row r="15" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
       <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
+      <c r="C15" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D15" s="8">
+        <v>1</v>
+      </c>
+      <c r="E15" s="9">
+        <v>1</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I15" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J15" s="9">
+        <v>16</v>
+      </c>
+      <c r="K15" s="9">
+        <v>100</v>
+      </c>
+      <c r="L15" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M15" s="18"/>
       <c r="N15" s="18"/>
       <c r="O15" s="18"/>
@@ -3006,18 +3268,40 @@
       <c r="S15" s="19"/>
     </row>
     <row r="16" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
       <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
+      <c r="C16" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" s="8">
+        <v>1</v>
+      </c>
+      <c r="E16" s="9">
+        <v>1</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I16" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J16" s="9">
+        <v>16</v>
+      </c>
+      <c r="K16" s="9">
+        <v>100</v>
+      </c>
+      <c r="L16" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M16" s="18"/>
       <c r="N16" s="18"/>
       <c r="O16" s="18"/>
@@ -3027,18 +3311,40 @@
       <c r="S16" s="19"/>
     </row>
     <row r="17" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
       <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="9"/>
-      <c r="L17" s="9"/>
+      <c r="C17" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" s="8">
+        <v>1</v>
+      </c>
+      <c r="E17" s="9">
+        <v>1</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I17" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J17" s="9">
+        <v>16</v>
+      </c>
+      <c r="K17" s="9">
+        <v>100</v>
+      </c>
+      <c r="L17" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M17" s="18"/>
       <c r="N17" s="18"/>
       <c r="O17" s="18"/>
@@ -3048,18 +3354,40 @@
       <c r="S17" s="19"/>
     </row>
     <row r="18" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2"/>
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
       <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
+      <c r="C18" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="8">
+        <v>1</v>
+      </c>
+      <c r="E18" s="9">
+        <v>1</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I18" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J18" s="9">
+        <v>16</v>
+      </c>
+      <c r="K18" s="9">
+        <v>100</v>
+      </c>
+      <c r="L18" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M18" s="18"/>
       <c r="N18" s="18"/>
       <c r="O18" s="18"/>
@@ -3069,18 +3397,40 @@
       <c r="S18" s="19"/>
     </row>
     <row r="19" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="2"/>
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
       <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="9"/>
+      <c r="C19" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D19" s="8">
+        <v>1</v>
+      </c>
+      <c r="E19" s="9">
+        <v>1</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I19" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J19" s="9">
+        <v>16</v>
+      </c>
+      <c r="K19" s="9">
+        <v>100</v>
+      </c>
+      <c r="L19" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M19" s="18"/>
       <c r="N19" s="18"/>
       <c r="O19" s="18"/>

</xml_diff>

<commit_message>
added train results 13 to 23, for models version 10 and 11
</commit_message>
<xml_diff>
--- a/work.xlsx
+++ b/work.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\iman_heydardoost\research_papers\dental_paper_1\Dental-XRay-YOLO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F7D218-9DAA-402A-8E04-F6528BAC2CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21140C46-26BE-4815-963A-15782968E170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="660" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dataset" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="122">
   <si>
     <t>number of models in series</t>
   </si>
@@ -404,6 +404,24 @@
   </si>
   <si>
     <t>extra large</t>
+  </si>
+  <si>
+    <t>YOLOv11</t>
+  </si>
+  <si>
+    <t>14/6/2026</t>
+  </si>
+  <si>
+    <t>15/6/2026</t>
+  </si>
+  <si>
+    <t>16/6/2026</t>
+  </si>
+  <si>
+    <t>YOLOv12</t>
+  </si>
+  <si>
+    <t>17/6/2026</t>
   </si>
 </sst>
 </file>
@@ -2569,7 +2587,7 @@
         <v>0.44085999999999997</v>
       </c>
       <c r="Q3" s="18">
-        <f t="shared" ref="Q3:Q13" si="0">2*(O3*P3)/(O3+P3)</f>
+        <f t="shared" ref="Q3:Q24" si="0">2*(O3*P3)/(O3+P3)</f>
         <v>0.48310328151277737</v>
       </c>
       <c r="R3" s="18">
@@ -3216,19 +3234,36 @@
       <c r="L14" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M14" s="18"/>
-      <c r="N14" s="18"/>
-      <c r="O14" s="18"/>
-      <c r="P14" s="18"/>
-      <c r="Q14" s="18"/>
-      <c r="R14" s="18"/>
-      <c r="S14" s="19"/>
+      <c r="M14" s="18">
+        <v>0.47465000000000002</v>
+      </c>
+      <c r="N14" s="18">
+        <v>0.24507999999999999</v>
+      </c>
+      <c r="O14" s="18">
+        <v>0.50299000000000005</v>
+      </c>
+      <c r="P14" s="18">
+        <v>0.51041999999999998</v>
+      </c>
+      <c r="Q14" s="18">
+        <f t="shared" si="0"/>
+        <v>0.50667776280084087</v>
+      </c>
+      <c r="R14" s="18">
+        <v>0.4</v>
+      </c>
+      <c r="S14" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="15" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="B15" s="8"/>
+      <c r="B15" s="24">
+        <v>46301</v>
+      </c>
       <c r="C15" s="8" t="s">
         <v>97</v>
       </c>
@@ -3259,19 +3294,36 @@
       <c r="L15" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M15" s="18"/>
-      <c r="N15" s="18"/>
-      <c r="O15" s="18"/>
-      <c r="P15" s="18"/>
-      <c r="Q15" s="18"/>
-      <c r="R15" s="18"/>
-      <c r="S15" s="19"/>
+      <c r="M15" s="18">
+        <v>0.52751999999999999</v>
+      </c>
+      <c r="N15" s="18">
+        <v>0.28743000000000002</v>
+      </c>
+      <c r="O15" s="18">
+        <v>0.53896999999999995</v>
+      </c>
+      <c r="P15" s="18">
+        <v>0.53866999999999998</v>
+      </c>
+      <c r="Q15" s="18">
+        <f t="shared" si="0"/>
+        <v>0.53881995824208451</v>
+      </c>
+      <c r="R15" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="S15" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="16" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="B16" s="8"/>
+      <c r="B16" s="24">
+        <v>46332</v>
+      </c>
       <c r="C16" s="8" t="s">
         <v>97</v>
       </c>
@@ -3302,19 +3354,36 @@
       <c r="L16" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M16" s="18"/>
-      <c r="N16" s="18"/>
-      <c r="O16" s="18"/>
-      <c r="P16" s="18"/>
-      <c r="Q16" s="18"/>
-      <c r="R16" s="18"/>
-      <c r="S16" s="19"/>
+      <c r="M16" s="18">
+        <v>0.54427999999999999</v>
+      </c>
+      <c r="N16" s="18">
+        <v>0.30532999999999999</v>
+      </c>
+      <c r="O16" s="18">
+        <v>0.56603000000000003</v>
+      </c>
+      <c r="P16" s="18">
+        <v>0.54644999999999999</v>
+      </c>
+      <c r="Q16" s="18">
+        <f t="shared" si="0"/>
+        <v>0.55606769290234426</v>
+      </c>
+      <c r="R16" s="18">
+        <v>1.4</v>
+      </c>
+      <c r="S16" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="17" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>16</v>
       </c>
-      <c r="B17" s="8"/>
+      <c r="B17" s="24">
+        <v>46362</v>
+      </c>
       <c r="C17" s="8" t="s">
         <v>97</v>
       </c>
@@ -3345,19 +3414,36 @@
       <c r="L17" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M17" s="18"/>
-      <c r="N17" s="18"/>
-      <c r="O17" s="18"/>
-      <c r="P17" s="18"/>
-      <c r="Q17" s="18"/>
-      <c r="R17" s="18"/>
-      <c r="S17" s="19"/>
+      <c r="M17" s="18">
+        <v>0.55201</v>
+      </c>
+      <c r="N17" s="18">
+        <v>0.30665999999999999</v>
+      </c>
+      <c r="O17" s="18">
+        <v>0.58487999999999996</v>
+      </c>
+      <c r="P17" s="18">
+        <v>0.55086000000000002</v>
+      </c>
+      <c r="Q17" s="18">
+        <f>2*(O17*P17)/(O17+P17)</f>
+        <v>0.56736048180041199</v>
+      </c>
+      <c r="R17" s="18">
+        <v>1.5</v>
+      </c>
+      <c r="S17" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="18" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>17</v>
       </c>
-      <c r="B18" s="8"/>
+      <c r="B18" s="24">
+        <v>46362</v>
+      </c>
       <c r="C18" s="8" t="s">
         <v>97</v>
       </c>
@@ -3388,19 +3474,36 @@
       <c r="L18" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M18" s="18"/>
-      <c r="N18" s="18"/>
-      <c r="O18" s="18"/>
-      <c r="P18" s="18"/>
-      <c r="Q18" s="18"/>
-      <c r="R18" s="18"/>
-      <c r="S18" s="19"/>
+      <c r="M18" s="18">
+        <v>0.56154000000000004</v>
+      </c>
+      <c r="N18" s="18">
+        <v>0.31391999999999998</v>
+      </c>
+      <c r="O18" s="18">
+        <v>0.59721000000000002</v>
+      </c>
+      <c r="P18" s="18">
+        <v>0.55179999999999996</v>
+      </c>
+      <c r="Q18" s="18">
+        <f t="shared" si="0"/>
+        <v>0.57360767617340136</v>
+      </c>
+      <c r="R18" s="18">
+        <v>2.1</v>
+      </c>
+      <c r="S18" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="19" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>18</v>
       </c>
-      <c r="B19" s="8"/>
+      <c r="B19" s="24">
+        <v>46362</v>
+      </c>
       <c r="C19" s="8" t="s">
         <v>97</v>
       </c>
@@ -3431,132 +3534,366 @@
       <c r="L19" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M19" s="18"/>
-      <c r="N19" s="18"/>
-      <c r="O19" s="18"/>
-      <c r="P19" s="18"/>
-      <c r="Q19" s="18"/>
-      <c r="R19" s="18"/>
-      <c r="S19" s="19"/>
+      <c r="M19" s="18">
+        <v>0.56569999999999998</v>
+      </c>
+      <c r="N19" s="18">
+        <v>0.32196999999999998</v>
+      </c>
+      <c r="O19" s="18">
+        <v>0.59689000000000003</v>
+      </c>
+      <c r="P19" s="18">
+        <v>0.55559999999999998</v>
+      </c>
+      <c r="Q19" s="18">
+        <f t="shared" si="0"/>
+        <v>0.57550535622868748</v>
+      </c>
+      <c r="R19" s="18">
+        <v>2.5</v>
+      </c>
+      <c r="S19" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="20" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="2"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-      <c r="L20" s="9"/>
-      <c r="M20" s="18"/>
-      <c r="N20" s="18"/>
-      <c r="O20" s="18"/>
-      <c r="P20" s="18"/>
-      <c r="Q20" s="18"/>
-      <c r="R20" s="18"/>
-      <c r="S20" s="19"/>
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D20" s="8">
+        <v>1</v>
+      </c>
+      <c r="E20" s="9">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I20" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J20" s="9">
+        <v>16</v>
+      </c>
+      <c r="K20" s="9">
+        <v>100</v>
+      </c>
+      <c r="L20" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M20" s="18">
+        <v>0.48680000000000001</v>
+      </c>
+      <c r="N20" s="18">
+        <v>0.24876000000000001</v>
+      </c>
+      <c r="O20" s="18">
+        <v>0.52778000000000003</v>
+      </c>
+      <c r="P20" s="18">
+        <v>0.51315999999999995</v>
+      </c>
+      <c r="Q20" s="18">
+        <f t="shared" si="0"/>
+        <v>0.52036733106615174</v>
+      </c>
+      <c r="R20" s="18">
+        <v>0.3</v>
+      </c>
+      <c r="S20" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="21" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="2"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
-      <c r="L21" s="9"/>
-      <c r="M21" s="18"/>
-      <c r="N21" s="18"/>
-      <c r="O21" s="18"/>
-      <c r="P21" s="18"/>
-      <c r="Q21" s="18"/>
-      <c r="R21" s="18"/>
-      <c r="S21" s="19"/>
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D21" s="8">
+        <v>1</v>
+      </c>
+      <c r="E21" s="9">
+        <v>1</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I21" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J21" s="9">
+        <v>16</v>
+      </c>
+      <c r="K21" s="9">
+        <v>100</v>
+      </c>
+      <c r="L21" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M21" s="18">
+        <v>0.53566000000000003</v>
+      </c>
+      <c r="N21" s="18">
+        <v>0.28981000000000001</v>
+      </c>
+      <c r="O21" s="18">
+        <v>0.54568000000000005</v>
+      </c>
+      <c r="P21" s="18">
+        <v>0.54800000000000004</v>
+      </c>
+      <c r="Q21" s="18">
+        <f t="shared" si="0"/>
+        <v>0.54683753931680212</v>
+      </c>
+      <c r="R21" s="18">
+        <v>0.6</v>
+      </c>
+      <c r="S21" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="22" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="2"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="9"/>
-      <c r="L22" s="9"/>
-      <c r="M22" s="18"/>
-      <c r="N22" s="18"/>
-      <c r="O22" s="18"/>
-      <c r="P22" s="18"/>
-      <c r="Q22" s="18"/>
-      <c r="R22" s="18"/>
-      <c r="S22" s="19"/>
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D22" s="8">
+        <v>1</v>
+      </c>
+      <c r="E22" s="9">
+        <v>1</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I22" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J22" s="9">
+        <v>16</v>
+      </c>
+      <c r="K22" s="9">
+        <v>100</v>
+      </c>
+      <c r="L22" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M22" s="18">
+        <v>0.54627999999999999</v>
+      </c>
+      <c r="N22" s="18">
+        <v>0.30147000000000002</v>
+      </c>
+      <c r="O22" s="18">
+        <v>0.58565</v>
+      </c>
+      <c r="P22" s="18">
+        <v>0.56564000000000003</v>
+      </c>
+      <c r="Q22" s="18">
+        <f t="shared" si="0"/>
+        <v>0.57547110806139201</v>
+      </c>
+      <c r="R22" s="18">
+        <v>1.2</v>
+      </c>
+      <c r="S22" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="23" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="2"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="9"/>
-      <c r="L23" s="9"/>
-      <c r="M23" s="18"/>
-      <c r="N23" s="18"/>
-      <c r="O23" s="18"/>
-      <c r="P23" s="18"/>
-      <c r="Q23" s="18"/>
-      <c r="R23" s="18"/>
-      <c r="S23" s="19"/>
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D23" s="8">
+        <v>1</v>
+      </c>
+      <c r="E23" s="9">
+        <v>1</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I23" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J23" s="9">
+        <v>16</v>
+      </c>
+      <c r="K23" s="9">
+        <v>100</v>
+      </c>
+      <c r="L23" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M23" s="18">
+        <v>0.55788000000000004</v>
+      </c>
+      <c r="N23" s="18">
+        <v>0.31286999999999998</v>
+      </c>
+      <c r="O23" s="18">
+        <v>0.58509999999999995</v>
+      </c>
+      <c r="P23" s="18">
+        <v>0.56116999999999995</v>
+      </c>
+      <c r="Q23" s="18">
+        <f>2*(O23*P23)/(O23+P23)</f>
+        <v>0.57288521378034829</v>
+      </c>
+      <c r="R23" s="18">
+        <v>1.5</v>
+      </c>
+      <c r="S23" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="24" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="2"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
-      <c r="M24" s="18"/>
-      <c r="N24" s="18"/>
-      <c r="O24" s="18"/>
-      <c r="P24" s="18"/>
-      <c r="Q24" s="18"/>
-      <c r="R24" s="18"/>
-      <c r="S24" s="19"/>
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D24" s="8">
+        <v>1</v>
+      </c>
+      <c r="E24" s="9">
+        <v>1</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I24" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J24" s="9">
+        <v>16</v>
+      </c>
+      <c r="K24" s="9">
+        <v>100</v>
+      </c>
+      <c r="L24" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M24" s="18">
+        <v>0.57747000000000004</v>
+      </c>
+      <c r="N24" s="18">
+        <v>0.33184999999999998</v>
+      </c>
+      <c r="O24" s="18">
+        <v>0.61217999999999995</v>
+      </c>
+      <c r="P24" s="18">
+        <v>0.57835999999999999</v>
+      </c>
+      <c r="Q24" s="18">
+        <f t="shared" si="0"/>
+        <v>0.59478963293967435</v>
+      </c>
+      <c r="R24" s="18">
+        <v>2.6</v>
+      </c>
+      <c r="S24" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="25" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="2"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
-      <c r="K25" s="9"/>
-      <c r="L25" s="9"/>
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D25" s="8">
+        <v>1</v>
+      </c>
+      <c r="E25" s="9">
+        <v>1</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I25" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J25" s="9">
+        <v>16</v>
+      </c>
+      <c r="K25" s="9">
+        <v>100</v>
+      </c>
+      <c r="L25" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M25" s="18"/>
       <c r="N25" s="18"/>
       <c r="O25" s="18"/>
@@ -3566,18 +3903,42 @@
       <c r="S25" s="19"/>
     </row>
     <row r="26" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="2"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
-      <c r="K26" s="9"/>
-      <c r="L26" s="9"/>
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D26" s="8">
+        <v>1</v>
+      </c>
+      <c r="E26" s="9">
+        <v>1</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I26" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J26" s="9">
+        <v>16</v>
+      </c>
+      <c r="K26" s="9">
+        <v>100</v>
+      </c>
+      <c r="L26" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M26" s="18"/>
       <c r="N26" s="18"/>
       <c r="O26" s="18"/>
@@ -3587,18 +3948,42 @@
       <c r="S26" s="19"/>
     </row>
     <row r="27" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="2"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="9"/>
-      <c r="L27" s="9"/>
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D27" s="8">
+        <v>1</v>
+      </c>
+      <c r="E27" s="9">
+        <v>1</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I27" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J27" s="9">
+        <v>16</v>
+      </c>
+      <c r="K27" s="9">
+        <v>100</v>
+      </c>
+      <c r="L27" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M27" s="18"/>
       <c r="N27" s="18"/>
       <c r="O27" s="18"/>
@@ -3608,18 +3993,40 @@
       <c r="S27" s="19"/>
     </row>
     <row r="28" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="2"/>
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
       <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
-      <c r="K28" s="9"/>
-      <c r="L28" s="9"/>
+      <c r="C28" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D28" s="8">
+        <v>1</v>
+      </c>
+      <c r="E28" s="9">
+        <v>1</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I28" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J28" s="9">
+        <v>16</v>
+      </c>
+      <c r="K28" s="9">
+        <v>100</v>
+      </c>
+      <c r="L28" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M28" s="18"/>
       <c r="N28" s="18"/>
       <c r="O28" s="18"/>
@@ -3629,18 +4036,40 @@
       <c r="S28" s="19"/>
     </row>
     <row r="29" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="2"/>
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
       <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="9"/>
-      <c r="K29" s="9"/>
-      <c r="L29" s="9"/>
+      <c r="C29" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D29" s="8">
+        <v>1</v>
+      </c>
+      <c r="E29" s="9">
+        <v>1</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="H29" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I29" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J29" s="9">
+        <v>16</v>
+      </c>
+      <c r="K29" s="9">
+        <v>100</v>
+      </c>
+      <c r="L29" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M29" s="18"/>
       <c r="N29" s="18"/>
       <c r="O29" s="18"/>

</xml_diff>

<commit_message>
added train results 24 to 28, for model version 12
</commit_message>
<xml_diff>
--- a/work.xlsx
+++ b/work.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\iman_heydardoost\research_papers\dental_paper_1\Dental-XRay-YOLO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21140C46-26BE-4815-963A-15782968E170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED26B495-D065-4B71-BA59-5A23E409FDF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="660" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dataset" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="125">
   <si>
     <t>number of models in series</t>
   </si>
@@ -422,6 +422,15 @@
   </si>
   <si>
     <t>17/6/2026</t>
+  </si>
+  <si>
+    <t>19/6/2026</t>
+  </si>
+  <si>
+    <t>20/6/2026</t>
+  </si>
+  <si>
+    <t>YOLOv13</t>
   </si>
 </sst>
 </file>
@@ -2587,7 +2596,7 @@
         <v>0.44085999999999997</v>
       </c>
       <c r="Q3" s="18">
-        <f t="shared" ref="Q3:Q24" si="0">2*(O3*P3)/(O3+P3)</f>
+        <f t="shared" ref="Q3:Q29" si="0">2*(O3*P3)/(O3+P3)</f>
         <v>0.48310328151277737</v>
       </c>
       <c r="R3" s="18">
@@ -3894,13 +3903,28 @@
       <c r="L25" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M25" s="18"/>
-      <c r="N25" s="18"/>
-      <c r="O25" s="18"/>
-      <c r="P25" s="18"/>
-      <c r="Q25" s="18"/>
-      <c r="R25" s="18"/>
-      <c r="S25" s="19"/>
+      <c r="M25" s="18">
+        <v>0.50438000000000005</v>
+      </c>
+      <c r="N25" s="18">
+        <v>0.26529999999999998</v>
+      </c>
+      <c r="O25" s="18">
+        <v>0.51512000000000002</v>
+      </c>
+      <c r="P25" s="18">
+        <v>0.52988999999999997</v>
+      </c>
+      <c r="Q25" s="18">
+        <f t="shared" si="0"/>
+        <v>0.52240062162084577</v>
+      </c>
+      <c r="R25" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="S25" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="26" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
@@ -3939,13 +3963,28 @@
       <c r="L26" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M26" s="18"/>
-      <c r="N26" s="18"/>
-      <c r="O26" s="18"/>
-      <c r="P26" s="18"/>
-      <c r="Q26" s="18"/>
-      <c r="R26" s="18"/>
-      <c r="S26" s="19"/>
+      <c r="M26" s="18">
+        <v>0.54124000000000005</v>
+      </c>
+      <c r="N26" s="18">
+        <v>0.29425000000000001</v>
+      </c>
+      <c r="O26" s="18">
+        <v>0.59186000000000005</v>
+      </c>
+      <c r="P26" s="18">
+        <v>0.54574999999999996</v>
+      </c>
+      <c r="Q26" s="18">
+        <f t="shared" si="0"/>
+        <v>0.56787052680619887</v>
+      </c>
+      <c r="R26" s="18">
+        <v>0.8</v>
+      </c>
+      <c r="S26" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="27" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
@@ -3984,19 +4023,36 @@
       <c r="L27" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M27" s="18"/>
-      <c r="N27" s="18"/>
-      <c r="O27" s="18"/>
-      <c r="P27" s="18"/>
-      <c r="Q27" s="18"/>
-      <c r="R27" s="18"/>
-      <c r="S27" s="19"/>
+      <c r="M27" s="18">
+        <v>0.55291999999999997</v>
+      </c>
+      <c r="N27" s="18">
+        <v>0.30829000000000001</v>
+      </c>
+      <c r="O27" s="18">
+        <v>0.60165999999999997</v>
+      </c>
+      <c r="P27" s="18">
+        <v>0.55215999999999998</v>
+      </c>
+      <c r="Q27" s="18">
+        <f t="shared" si="0"/>
+        <v>0.5758482009325544</v>
+      </c>
+      <c r="R27" s="18">
+        <v>1.7</v>
+      </c>
+      <c r="S27" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="28" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>27</v>
       </c>
-      <c r="B28" s="8"/>
+      <c r="B28" s="8" t="s">
+        <v>121</v>
+      </c>
       <c r="C28" s="8" t="s">
         <v>97</v>
       </c>
@@ -4027,19 +4083,36 @@
       <c r="L28" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M28" s="18"/>
-      <c r="N28" s="18"/>
-      <c r="O28" s="18"/>
-      <c r="P28" s="18"/>
-      <c r="Q28" s="18"/>
-      <c r="R28" s="18"/>
-      <c r="S28" s="19"/>
+      <c r="M28" s="18">
+        <v>0.55286000000000002</v>
+      </c>
+      <c r="N28" s="18">
+        <v>0.30885000000000001</v>
+      </c>
+      <c r="O28" s="18">
+        <v>0.57791999999999999</v>
+      </c>
+      <c r="P28" s="18">
+        <v>0.55991999999999997</v>
+      </c>
+      <c r="Q28" s="18">
+        <f>2*(O28*P28)/(O28+P28)</f>
+        <v>0.56877762497363415</v>
+      </c>
+      <c r="R28" s="18">
+        <v>2.5</v>
+      </c>
+      <c r="S28" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="29" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>28</v>
       </c>
-      <c r="B29" s="8"/>
+      <c r="B29" s="8" t="s">
+        <v>122</v>
+      </c>
       <c r="C29" s="8" t="s">
         <v>97</v>
       </c>
@@ -4070,27 +4143,66 @@
       <c r="L29" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="M29" s="18"/>
-      <c r="N29" s="18"/>
-      <c r="O29" s="18"/>
-      <c r="P29" s="18"/>
-      <c r="Q29" s="18"/>
-      <c r="R29" s="18"/>
-      <c r="S29" s="19"/>
+      <c r="M29" s="18">
+        <v>0.56076000000000004</v>
+      </c>
+      <c r="N29" s="18">
+        <v>0.31581999999999999</v>
+      </c>
+      <c r="O29" s="18">
+        <v>0.59226999999999996</v>
+      </c>
+      <c r="P29" s="18">
+        <v>0.56588000000000005</v>
+      </c>
+      <c r="Q29" s="18">
+        <f t="shared" si="0"/>
+        <v>0.57877433423995162</v>
+      </c>
+      <c r="R29" s="18">
+        <v>4.2</v>
+      </c>
+      <c r="S29" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="30" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="2"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="9"/>
-      <c r="K30" s="9"/>
-      <c r="L30" s="9"/>
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D30" s="8">
+        <v>1</v>
+      </c>
+      <c r="E30" s="9">
+        <v>1</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I30" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J30" s="9">
+        <v>16</v>
+      </c>
+      <c r="K30" s="9">
+        <v>100</v>
+      </c>
+      <c r="L30" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M30" s="18"/>
       <c r="N30" s="18"/>
       <c r="O30" s="18"/>
@@ -4100,18 +4212,40 @@
       <c r="S30" s="19"/>
     </row>
     <row r="31" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="2"/>
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
       <c r="B31" s="8"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="9"/>
-      <c r="K31" s="9"/>
-      <c r="L31" s="9"/>
+      <c r="C31" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31" s="8">
+        <v>1</v>
+      </c>
+      <c r="E31" s="9">
+        <v>1</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I31" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J31" s="9">
+        <v>16</v>
+      </c>
+      <c r="K31" s="9">
+        <v>100</v>
+      </c>
+      <c r="L31" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M31" s="18"/>
       <c r="N31" s="18"/>
       <c r="O31" s="18"/>
@@ -4121,18 +4255,40 @@
       <c r="S31" s="19"/>
     </row>
     <row r="32" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="2"/>
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
       <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="9"/>
-      <c r="H32" s="9"/>
-      <c r="I32" s="9"/>
-      <c r="J32" s="9"/>
-      <c r="K32" s="9"/>
-      <c r="L32" s="9"/>
+      <c r="C32" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D32" s="8">
+        <v>1</v>
+      </c>
+      <c r="E32" s="9">
+        <v>1</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I32" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J32" s="9">
+        <v>16</v>
+      </c>
+      <c r="K32" s="9">
+        <v>100</v>
+      </c>
+      <c r="L32" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M32" s="18"/>
       <c r="N32" s="18"/>
       <c r="O32" s="18"/>
@@ -4142,18 +4298,40 @@
       <c r="S32" s="19"/>
     </row>
     <row r="33" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="2"/>
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
       <c r="B33" s="8"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-      <c r="G33" s="9"/>
-      <c r="H33" s="9"/>
-      <c r="I33" s="9"/>
-      <c r="J33" s="9"/>
-      <c r="K33" s="9"/>
-      <c r="L33" s="9"/>
+      <c r="C33" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D33" s="8">
+        <v>1</v>
+      </c>
+      <c r="E33" s="9">
+        <v>1</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="H33" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I33" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J33" s="9">
+        <v>16</v>
+      </c>
+      <c r="K33" s="9">
+        <v>100</v>
+      </c>
+      <c r="L33" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="M33" s="18"/>
       <c r="N33" s="18"/>
       <c r="O33" s="18"/>

</xml_diff>

<commit_message>
added train results 33 to 37, for model version 26
</commit_message>
<xml_diff>
--- a/work.xlsx
+++ b/work.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\iman_heydardoost\research_papers\dental_paper_1\Dental-XRay-YOLO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED26B495-D065-4B71-BA59-5A23E409FDF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58DADD0A-D103-45A6-8EA8-9E0AE23B6474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="660" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="129">
   <si>
     <t>number of models in series</t>
   </si>
@@ -427,10 +427,22 @@
     <t>19/6/2026</t>
   </si>
   <si>
-    <t>20/6/2026</t>
-  </si>
-  <si>
     <t>YOLOv13</t>
+  </si>
+  <si>
+    <t>YOLOv26</t>
+  </si>
+  <si>
+    <t>24/6/2026</t>
+  </si>
+  <si>
+    <t>25/6/2026</t>
+  </si>
+  <si>
+    <t>26/6/2026</t>
+  </si>
+  <si>
+    <t>27/6/2026</t>
   </si>
 </sst>
 </file>
@@ -2596,7 +2608,7 @@
         <v>0.44085999999999997</v>
       </c>
       <c r="Q3" s="18">
-        <f t="shared" ref="Q3:Q29" si="0">2*(O3*P3)/(O3+P3)</f>
+        <f t="shared" ref="Q3:Q38" si="0">2*(O3*P3)/(O3+P3)</f>
         <v>0.48310328151277737</v>
       </c>
       <c r="R3" s="18">
@@ -4170,9 +4182,7 @@
       <c r="A30" s="2">
         <v>29</v>
       </c>
-      <c r="B30" s="8" t="s">
-        <v>123</v>
-      </c>
+      <c r="B30" s="8"/>
       <c r="C30" s="8" t="s">
         <v>97</v>
       </c>
@@ -4183,7 +4193,7 @@
         <v>1</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G30" s="9" t="s">
         <v>37</v>
@@ -4226,7 +4236,7 @@
         <v>1</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G31" s="9" t="s">
         <v>102</v>
@@ -4269,7 +4279,7 @@
         <v>1</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G32" s="9" t="s">
         <v>106</v>
@@ -4312,7 +4322,7 @@
         <v>1</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G33" s="9" t="s">
         <v>107</v>
@@ -4341,109 +4351,304 @@
       <c r="S33" s="19"/>
     </row>
     <row r="34" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="2"/>
-      <c r="B34" s="8"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
-      <c r="I34" s="9"/>
-      <c r="J34" s="9"/>
-      <c r="K34" s="9"/>
-      <c r="L34" s="9"/>
-      <c r="M34" s="18"/>
-      <c r="N34" s="18"/>
-      <c r="O34" s="18"/>
-      <c r="P34" s="18"/>
-      <c r="Q34" s="18"/>
-      <c r="R34" s="18"/>
-      <c r="S34" s="19"/>
+      <c r="A34" s="2">
+        <v>33</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D34" s="8">
+        <v>1</v>
+      </c>
+      <c r="E34" s="9">
+        <v>1</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H34" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I34" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J34" s="9">
+        <v>16</v>
+      </c>
+      <c r="K34" s="9">
+        <v>100</v>
+      </c>
+      <c r="L34" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M34" s="18">
+        <v>0.45791999999999999</v>
+      </c>
+      <c r="N34" s="18">
+        <v>0.23643</v>
+      </c>
+      <c r="O34" s="18">
+        <v>0.47811999999999999</v>
+      </c>
+      <c r="P34" s="18">
+        <v>0.48646</v>
+      </c>
+      <c r="Q34" s="18">
+        <f t="shared" si="0"/>
+        <v>0.48225394513674347</v>
+      </c>
+      <c r="R34" s="18">
+        <v>0.7</v>
+      </c>
+      <c r="S34" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="35" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="2"/>
-      <c r="B35" s="8"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="9"/>
-      <c r="K35" s="9"/>
-      <c r="L35" s="9"/>
-      <c r="M35" s="18"/>
-      <c r="N35" s="18"/>
-      <c r="O35" s="18"/>
-      <c r="P35" s="18"/>
-      <c r="Q35" s="18"/>
-      <c r="R35" s="18"/>
-      <c r="S35" s="19"/>
+      <c r="A35" s="2">
+        <v>34</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D35" s="8">
+        <v>1</v>
+      </c>
+      <c r="E35" s="9">
+        <v>1</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="H35" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I35" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J35" s="9">
+        <v>16</v>
+      </c>
+      <c r="K35" s="9">
+        <v>100</v>
+      </c>
+      <c r="L35" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M35" s="18">
+        <v>0.50834000000000001</v>
+      </c>
+      <c r="N35" s="18">
+        <v>0.27543000000000001</v>
+      </c>
+      <c r="O35" s="18">
+        <v>0.52737000000000001</v>
+      </c>
+      <c r="P35" s="18">
+        <v>0.52800999999999998</v>
+      </c>
+      <c r="Q35" s="18">
+        <f t="shared" si="0"/>
+        <v>0.52768980594667325</v>
+      </c>
+      <c r="R35" s="18">
+        <v>0.9</v>
+      </c>
+      <c r="S35" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="36" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="2"/>
-      <c r="B36" s="8"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="9"/>
-      <c r="J36" s="9"/>
-      <c r="K36" s="9"/>
-      <c r="L36" s="9"/>
-      <c r="M36" s="18"/>
-      <c r="N36" s="18"/>
-      <c r="O36" s="18"/>
-      <c r="P36" s="18"/>
-      <c r="Q36" s="18"/>
-      <c r="R36" s="18"/>
-      <c r="S36" s="19"/>
+      <c r="A36" s="2">
+        <v>35</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D36" s="8">
+        <v>1</v>
+      </c>
+      <c r="E36" s="9">
+        <v>1</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H36" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I36" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J36" s="9">
+        <v>16</v>
+      </c>
+      <c r="K36" s="9">
+        <v>100</v>
+      </c>
+      <c r="L36" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M36" s="18">
+        <v>0.5333</v>
+      </c>
+      <c r="N36" s="18">
+        <v>0.29421999999999998</v>
+      </c>
+      <c r="O36" s="18">
+        <v>0.54515000000000002</v>
+      </c>
+      <c r="P36" s="18">
+        <v>0.54183000000000003</v>
+      </c>
+      <c r="Q36" s="18">
+        <f t="shared" si="0"/>
+        <v>0.54348492980551621</v>
+      </c>
+      <c r="R36" s="18">
+        <v>1.6</v>
+      </c>
+      <c r="S36" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="37" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="2"/>
-      <c r="B37" s="8"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
-      <c r="H37" s="9"/>
-      <c r="I37" s="9"/>
-      <c r="J37" s="9"/>
-      <c r="K37" s="9"/>
-      <c r="L37" s="9"/>
-      <c r="M37" s="18"/>
-      <c r="N37" s="18"/>
-      <c r="O37" s="18"/>
-      <c r="P37" s="18"/>
-      <c r="Q37" s="18"/>
-      <c r="R37" s="18"/>
-      <c r="S37" s="19"/>
+      <c r="A37" s="2">
+        <v>36</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D37" s="8">
+        <v>1</v>
+      </c>
+      <c r="E37" s="9">
+        <v>1</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="H37" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I37" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J37" s="9">
+        <v>16</v>
+      </c>
+      <c r="K37" s="9">
+        <v>100</v>
+      </c>
+      <c r="L37" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M37" s="18">
+        <v>0.54261000000000004</v>
+      </c>
+      <c r="N37" s="18">
+        <v>0.29779</v>
+      </c>
+      <c r="O37" s="18">
+        <v>0.59194999999999998</v>
+      </c>
+      <c r="P37" s="18">
+        <v>0.54410999999999998</v>
+      </c>
+      <c r="Q37" s="18">
+        <f t="shared" si="0"/>
+        <v>0.56702271799024684</v>
+      </c>
+      <c r="R37" s="18">
+        <v>1.8</v>
+      </c>
+      <c r="S37" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="38" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="2"/>
-      <c r="B38" s="8"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="9"/>
-      <c r="I38" s="9"/>
-      <c r="J38" s="9"/>
-      <c r="K38" s="9"/>
-      <c r="L38" s="9"/>
-      <c r="M38" s="18"/>
-      <c r="N38" s="18"/>
-      <c r="O38" s="18"/>
-      <c r="P38" s="18"/>
-      <c r="Q38" s="18"/>
-      <c r="R38" s="18"/>
-      <c r="S38" s="19"/>
+      <c r="A38" s="2">
+        <v>37</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D38" s="8">
+        <v>1</v>
+      </c>
+      <c r="E38" s="9">
+        <v>1</v>
+      </c>
+      <c r="F38" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G38" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="H38" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I38" s="9">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J38" s="9">
+        <v>16</v>
+      </c>
+      <c r="K38" s="9">
+        <v>100</v>
+      </c>
+      <c r="L38" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M38" s="18">
+        <v>0.57818000000000003</v>
+      </c>
+      <c r="N38" s="18">
+        <v>0.32368000000000002</v>
+      </c>
+      <c r="O38" s="18">
+        <v>0.65951000000000004</v>
+      </c>
+      <c r="P38" s="18">
+        <v>0.55066999999999999</v>
+      </c>
+      <c r="Q38" s="18">
+        <f t="shared" si="0"/>
+        <v>0.60019562660100145</v>
+      </c>
+      <c r="R38" s="18">
+        <v>2.8</v>
+      </c>
+      <c r="S38" s="19">
+        <v>100</v>
+      </c>
     </row>
     <row r="39" spans="1:19" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>

</xml_diff>